<commit_message>
Add per-customer master data (contact person, billing phrase)
The user's real historical invoice archive (uploaded as reference)
showed that 担当者 and the closing phrase ("ご請求申し上げます。" vs
"ご注文を受付致します。") vary by client, not globally as previously
hardcoded — e.g. one client's invoices always list a different
contact person and use order-acceptance wording instead of billing
wording. Sending the wrong one would be an obvious, visible mistake
on a real client-facing document.

Adds a "顧客マスタ" sheet (customer_name -> contact, phrase) that
create_invoice_pdf now reads per customer, falling back to sane
defaults if the sheet or the customer's row is missing. Updated the
template and sample data to match.
</commit_message>
<xml_diff>
--- a/invoice_agent/invoice_template.xlsx
+++ b/invoice_agent/invoice_template.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="請求データ" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="顧客マスタ" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -189,6 +190,31 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>invoice_agent</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>「請求データ」シートの顧客名と一致させる</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>請求書右上に載る担当者名</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>請求書の本文。「下記の通り、ご請求申し上げます。」か「下記の通り、ご注文を受付致します。」など、顧客ごとに決まった文言があれば入力（空欄ならご請求申し上げます。になる）</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -633,4 +659,58 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>顧客名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>担当者</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>請求文言</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>（記入例）A社</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>辰巳</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>下記の通り、ご請求申し上げます。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Set Vastra's contact person to 竹田 in customer master
Also add Vastra as a customer master entry in the reusable
invoice_template.xlsx for future months.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/invoice_template.xlsx
+++ b/invoice_agent/invoice_template.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -709,6 +709,19 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Vastra</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>竹田</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Add WillWay's August invoice, rebalance item table columns
Long item names (like WillWay's report title) were overflowing the
70mm 項目 column; widened it to 83mm and trimmed the mostly-empty
数量 column to make room. Also brought invoice_template.xlsx's
customer master up to date with the 敬称 column and existing
customers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/invoice_template.xlsx
+++ b/invoice_agent/invoice_template.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -691,6 +691,11 @@
           <t>請求文言</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>敬称</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -708,6 +713,11 @@
           <t>下記の通り、ご請求申し上げます。</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>御中</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -720,7 +730,28 @@
           <t>竹田</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>御中</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>大谷　晃巨</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>竹田</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>様</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>